<commit_message>
add: include W04 assessment and challenge files for module 4
</commit_message>
<xml_diff>
--- a/01-essentials/material_curso/modulo-03/W03-Assessment.xlsx
+++ b/01-essentials/material_curso/modulo-03/W03-Assessment.xlsx
@@ -1,33 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18067"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nic\Documents\Freelance Training\Maquarie Uni\MOOCS\Assessments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jorge\Proyectos\ExcelLearning\01-essentials\material_curso\modulo-03\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24206998-9CEE-4975-A775-6A34BADC80E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10524"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="86">
   <si>
     <t>Student No</t>
   </si>
@@ -276,14 +286,24 @@
   </si>
   <si>
     <t>Last Modified:</t>
+  </si>
+  <si>
+    <t>sss</t>
+  </si>
+  <si>
+    <t>ss</t>
+  </si>
+  <si>
+    <t>ssssss</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="166" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -400,7 +420,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="3" applyFont="1" applyAlignment="1"/>
@@ -432,9 +452,6 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -451,20 +468,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -485,39 +514,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Information"/>
-      <sheetName val="Instructions"/>
-      <sheetName val="Labour Costs"/>
-      <sheetName val="Activity Based Costs"/>
-      <sheetName val="Cost Drivers"/>
-      <sheetName val="BOM"/>
-      <sheetName val="Product Costs"/>
-      <sheetName val="Inventory"/>
-      <sheetName val="Mark Sheet"/>
-      <sheetName val="Stats"/>
-      <sheetName val="Grade Book"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -816,71 +812,72 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U39"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
     <col min="4" max="18" width="5" style="7" customWidth="1"/>
-    <col min="19" max="20" width="6.33203125" style="7" customWidth="1"/>
+    <col min="19" max="19" width="15.7109375" style="7" customWidth="1"/>
+    <col min="20" max="20" width="11.5703125" style="7" customWidth="1"/>
     <col min="21" max="21" width="30" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="46.2" x14ac:dyDescent="0.85">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:21" ht="46.5" x14ac:dyDescent="0.7">
+      <c r="A1" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20"/>
-      <c r="T1" s="20"/>
-      <c r="U1" s="20"/>
-    </row>
-    <row r="3" spans="1:21" s="19" customFormat="1" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="21" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+    </row>
+    <row r="3" spans="1:21" s="18" customFormat="1" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="23">
         <v>42161</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="24"/>
-      <c r="R3" s="24"/>
-      <c r="S3" s="24"/>
-      <c r="T3" s="24"/>
-      <c r="U3" s="24"/>
-    </row>
-    <row r="4" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="20"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
+      <c r="U3" s="21"/>
+    </row>
+    <row r="4" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
@@ -901,65 +898,65 @@
       <c r="T4" s="8"/>
       <c r="U4" s="8"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="C5" s="15" t="s">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="C5" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="D5" s="16">
-        <v>2</v>
-      </c>
-      <c r="E5" s="16">
-        <v>2</v>
-      </c>
-      <c r="F5" s="16">
-        <v>2</v>
-      </c>
-      <c r="G5" s="16">
-        <v>2</v>
-      </c>
-      <c r="H5" s="16">
-        <v>1</v>
-      </c>
-      <c r="I5" s="16">
-        <v>1</v>
-      </c>
-      <c r="J5" s="16">
-        <v>1</v>
-      </c>
-      <c r="K5" s="16">
-        <v>1</v>
-      </c>
-      <c r="L5" s="16">
-        <v>1</v>
-      </c>
-      <c r="M5" s="16">
+      <c r="D5" s="15">
+        <v>2</v>
+      </c>
+      <c r="E5" s="15">
+        <v>2</v>
+      </c>
+      <c r="F5" s="15">
+        <v>2</v>
+      </c>
+      <c r="G5" s="15">
+        <v>2</v>
+      </c>
+      <c r="H5" s="15">
+        <v>1</v>
+      </c>
+      <c r="I5" s="15">
+        <v>1</v>
+      </c>
+      <c r="J5" s="15">
+        <v>1</v>
+      </c>
+      <c r="K5" s="15">
+        <v>1</v>
+      </c>
+      <c r="L5" s="15">
+        <v>1</v>
+      </c>
+      <c r="M5" s="15">
         <v>9</v>
       </c>
-      <c r="N5" s="16">
-        <v>7</v>
-      </c>
-      <c r="O5" s="16">
-        <v>3</v>
-      </c>
-      <c r="P5" s="16">
-        <v>3</v>
-      </c>
-      <c r="Q5" s="16">
-        <v>3</v>
-      </c>
-      <c r="R5" s="16">
-        <v>2</v>
-      </c>
-      <c r="S5" s="16">
+      <c r="N5" s="15">
+        <v>7</v>
+      </c>
+      <c r="O5" s="15">
+        <v>3</v>
+      </c>
+      <c r="P5" s="15">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="15">
+        <v>3</v>
+      </c>
+      <c r="R5" s="15">
+        <v>2</v>
+      </c>
+      <c r="S5" s="15">
         <f>SUM(D5:R5)</f>
         <v>40</v>
       </c>
-      <c r="T5" s="17">
-        <v>1</v>
-      </c>
-      <c r="U5" s="17"/>
-    </row>
-    <row r="6" spans="1:21" ht="66" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T5" s="16">
+        <v>1</v>
+      </c>
+      <c r="U5" s="16"/>
+    </row>
+    <row r="6" spans="1:21" ht="66" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>0</v>
       </c>
@@ -1024,7 +1021,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>158873</v>
       </c>
@@ -1084,12 +1081,12 @@
         <v>40</v>
       </c>
       <c r="T7" s="11">
-        <f>S7/$S$5</f>
+        <f t="shared" ref="T7:T36" si="0">S7/$S$5</f>
         <v>1</v>
       </c>
       <c r="U7" s="11"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>143319</v>
       </c>
@@ -1145,16 +1142,16 @@
         <v>2</v>
       </c>
       <c r="S8" s="7">
-        <f t="shared" ref="S8:S36" si="0">SUM(D8:R8)</f>
+        <f t="shared" ref="S8:S36" si="1">SUM(D8:R8)</f>
         <v>38</v>
       </c>
       <c r="T8" s="11">
-        <f>S8/$S$5</f>
+        <f t="shared" si="0"/>
         <v>0.95</v>
       </c>
       <c r="U8" s="11"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>146652</v>
       </c>
@@ -1210,16 +1207,16 @@
         <v>2</v>
       </c>
       <c r="S9" s="7">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="T9" s="24">
         <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-      <c r="T9" s="14">
-        <f>S9/$S$5</f>
         <v>0.92500000000000004</v>
       </c>
-      <c r="U9" s="14"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="U9" s="13"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>139986</v>
       </c>
@@ -1275,16 +1272,16 @@
         <v>1</v>
       </c>
       <c r="S10" s="7">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="T10" s="24">
         <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="T10" s="14">
-        <f>S10/$S$5</f>
         <v>0.6</v>
       </c>
       <c r="U10" s="11"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>137764</v>
       </c>
@@ -1340,16 +1337,16 @@
         <v>2</v>
       </c>
       <c r="S11" s="7">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="T11" s="11">
         <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-      <c r="T11" s="11">
-        <f>S11/$S$5</f>
         <v>0.85</v>
       </c>
       <c r="U11" s="11"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>151096</v>
       </c>
@@ -1405,16 +1402,16 @@
         <v>2</v>
       </c>
       <c r="S12" s="7">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="T12" s="11">
         <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-      <c r="T12" s="11">
-        <f>S12/$S$5</f>
         <v>1</v>
       </c>
       <c r="U12" s="11"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>185537</v>
       </c>
@@ -1470,16 +1467,16 @@
         <v>2</v>
       </c>
       <c r="S13" s="7">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+      <c r="T13" s="11">
         <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="T13" s="11">
-        <f>S13/$S$5</f>
         <v>0.72499999999999998</v>
       </c>
       <c r="U13" s="11"/>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>185537</v>
       </c>
@@ -1535,16 +1532,16 @@
         <v>2</v>
       </c>
       <c r="S14" s="7">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="T14" s="11">
         <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="T14" s="11">
-        <f>S14/$S$5</f>
         <v>0.47499999999999998</v>
       </c>
       <c r="U14" s="11"/>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>158873</v>
       </c>
@@ -1600,16 +1597,16 @@
         <v>2</v>
       </c>
       <c r="S15" s="7">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+      <c r="T15" s="11">
         <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="T15" s="11">
-        <f>S15/$S$5</f>
         <v>0.72499999999999998</v>
       </c>
       <c r="U15" s="11"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>182204</v>
       </c>
@@ -1665,16 +1662,16 @@
         <v>1</v>
       </c>
       <c r="S16" s="7">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="T16" s="11">
         <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="T16" s="11">
-        <f>S16/$S$5</f>
         <v>0.57499999999999996</v>
       </c>
       <c r="U16" s="11"/>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>172205</v>
       </c>
@@ -1730,16 +1727,16 @@
         <v>2</v>
       </c>
       <c r="S17" s="7">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="T17" s="11">
         <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-      <c r="T17" s="11">
-        <f>S17/$S$5</f>
         <v>0.9</v>
       </c>
       <c r="U17" s="11"/>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>176649</v>
       </c>
@@ -1795,16 +1792,16 @@
         <v>2</v>
       </c>
       <c r="S18" s="7">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="T18" s="11">
         <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-      <c r="T18" s="11">
-        <f>S18/$S$5</f>
         <v>0.95</v>
       </c>
       <c r="U18" s="11"/>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>156651</v>
       </c>
@@ -1860,16 +1857,16 @@
         <v>2</v>
       </c>
       <c r="S19" s="7">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="T19" s="11">
         <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-      <c r="T19" s="11">
-        <f>S19/$S$5</f>
         <v>0.95</v>
       </c>
       <c r="U19" s="11"/>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>174427</v>
       </c>
@@ -1925,16 +1922,16 @@
         <v>2</v>
       </c>
       <c r="S20" s="7">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="T20" s="11">
         <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-      <c r="T20" s="11">
-        <f>S20/$S$5</f>
         <v>0.875</v>
       </c>
       <c r="U20" s="11"/>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>154429</v>
       </c>
@@ -1990,16 +1987,16 @@
         <v>2</v>
       </c>
       <c r="S21" s="7">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="T21" s="11">
         <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-      <c r="T21" s="11">
-        <f>S21/$S$5</f>
         <v>0.875</v>
       </c>
       <c r="U21" s="11"/>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>166650</v>
       </c>
@@ -2055,16 +2052,16 @@
         <v>2</v>
       </c>
       <c r="S22" s="7">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+      <c r="T22" s="11">
         <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="T22" s="11">
-        <f>S22/$S$5</f>
         <v>0.7</v>
       </c>
       <c r="U22" s="11"/>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>152207</v>
       </c>
@@ -2120,16 +2117,16 @@
         <v>1</v>
       </c>
       <c r="S23" s="7">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="T23" s="11">
         <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="T23" s="11">
-        <f>S23/$S$5</f>
         <v>0.57499999999999996</v>
       </c>
       <c r="U23" s="11"/>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>163317</v>
       </c>
@@ -2185,16 +2182,16 @@
         <v>1</v>
       </c>
       <c r="S24" s="7">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="T24" s="11">
         <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="T24" s="11">
-        <f>S24/$S$5</f>
         <v>0.47499999999999998</v>
       </c>
       <c r="U24" s="11"/>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>156651</v>
       </c>
@@ -2250,16 +2247,16 @@
         <v>2</v>
       </c>
       <c r="S25" s="7">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="T25" s="11">
         <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-      <c r="T25" s="11">
-        <f>S25/$S$5</f>
         <v>0.85</v>
       </c>
       <c r="U25" s="11"/>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>138875</v>
       </c>
@@ -2315,16 +2312,16 @@
         <v>2</v>
       </c>
       <c r="S26" s="7">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+      <c r="T26" s="11">
         <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-      <c r="T26" s="11">
-        <f>S26/$S$5</f>
         <v>0.77500000000000002</v>
       </c>
       <c r="U26" s="11"/>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>178871</v>
       </c>
@@ -2380,16 +2377,16 @@
         <v>2</v>
       </c>
       <c r="S27" s="7">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+      <c r="T27" s="11">
         <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-      <c r="T27" s="11">
-        <f>S27/$S$5</f>
         <v>0.77500000000000002</v>
       </c>
       <c r="U27" s="11"/>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>157762</v>
       </c>
@@ -2445,16 +2442,16 @@
         <v>2</v>
       </c>
       <c r="S28" s="7">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+      <c r="T28" s="11">
         <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="T28" s="11">
-        <f>S28/$S$5</f>
         <v>0.82499999999999996</v>
       </c>
       <c r="U28" s="11"/>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>149985</v>
       </c>
@@ -2510,16 +2507,16 @@
         <v>1</v>
       </c>
       <c r="S29" s="7">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="T29" s="11">
         <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="T29" s="11">
-        <f>S29/$S$5</f>
         <v>0.57499999999999996</v>
       </c>
       <c r="U29" s="11"/>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>172205</v>
       </c>
@@ -2575,16 +2572,16 @@
         <v>2</v>
       </c>
       <c r="S30" s="7">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+      <c r="T30" s="11">
         <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="T30" s="11">
-        <f>S30/$S$5</f>
         <v>0.82499999999999996</v>
       </c>
       <c r="U30" s="11"/>
     </row>
-    <row r="31" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>158873</v>
       </c>
@@ -2640,18 +2637,18 @@
         <v>1</v>
       </c>
       <c r="S31" s="7">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="T31" s="11">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="T31" s="11">
-        <f>S31/$S$5</f>
         <v>0.35</v>
       </c>
-      <c r="U31" s="18" t="s">
+      <c r="U31" s="17" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>184426</v>
       </c>
@@ -2707,16 +2704,16 @@
         <v>2</v>
       </c>
       <c r="S32" s="7">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="T32" s="11">
         <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-      <c r="T32" s="11">
-        <f>S32/$S$5</f>
         <v>1</v>
       </c>
       <c r="U32" s="11"/>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>164428</v>
       </c>
@@ -2772,16 +2769,16 @@
         <v>1</v>
       </c>
       <c r="S33" s="7">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="T33" s="11">
         <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="T33" s="11">
-        <f>S33/$S$5</f>
         <v>0.65</v>
       </c>
       <c r="U33" s="11"/>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>141097</v>
       </c>
@@ -2837,16 +2834,16 @@
         <v>2</v>
       </c>
       <c r="S34" s="7">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="T34" s="11">
         <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-      <c r="T34" s="11">
-        <f>S34/$S$5</f>
         <v>0.9</v>
       </c>
       <c r="U34" s="11"/>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>146652</v>
       </c>
@@ -2902,16 +2899,16 @@
         <v>1</v>
       </c>
       <c r="S35" s="7">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="T35" s="11">
         <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="T35" s="11">
-        <f>S35/$S$5</f>
         <v>0.55000000000000004</v>
       </c>
       <c r="U35" s="11"/>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>171094</v>
       </c>
@@ -2967,16 +2964,16 @@
         <v>2</v>
       </c>
       <c r="S36" s="7">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="T36" s="11">
         <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-      <c r="T36" s="11">
-        <f>S36/$S$5</f>
         <v>0.95</v>
       </c>
       <c r="U36" s="11"/>
     </row>
-    <row r="38" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C38" s="9" t="s">
         <v>79</v>
       </c>
@@ -2995,7 +2992,7 @@
       <c r="P38" s="10"/>
       <c r="Q38" s="10"/>
       <c r="R38" s="10"/>
-      <c r="S38" s="13">
+      <c r="S38" s="27">
         <f>AVERAGE(S7:S36)</f>
         <v>30.866666666666667</v>
       </c>
@@ -3005,11 +3002,25 @@
       </c>
       <c r="U38" s="12"/>
     </row>
-    <row r="39" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E40" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:21" ht="91.5" x14ac:dyDescent="0.25">
+      <c r="H42" s="26" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>